<commit_message>
Correciones codigo. Modelo 1
</commit_message>
<xml_diff>
--- a/document/modelos.xlsx
+++ b/document/modelos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/camilaortiz/Dropbox/PEG/BigData/ProblemSet2_G10/document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F13796A5-2727-E74A-9C3B-5D152EF7AE7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78243E0C-97D6-D542-A07B-615E07474ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17400" yWindow="740" windowWidth="24960" windowHeight="16780" xr2:uid="{0E35A591-4511-AB40-9BF9-7C05772B802C}"/>
+    <workbookView xWindow="400" yWindow="740" windowWidth="11660" windowHeight="16780" xr2:uid="{0E35A591-4511-AB40-9BF9-7C05772B802C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t>Variables</t>
   </si>
@@ -80,9 +80,6 @@
     <t>N_pet</t>
   </si>
   <si>
-    <t>N_menpres</t>
-  </si>
-  <si>
     <t>N_mayor_dependiente</t>
   </si>
   <si>
@@ -123,6 +120,12 @@
   </si>
   <si>
     <t>Modelo 7</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>N_menores</t>
   </si>
 </sst>
 </file>
@@ -171,9 +174,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,40 +518,41 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="8" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
-      <c r="B2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="H2" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -560,16 +567,25 @@
       <c r="A7" t="s">
         <v>1</v>
       </c>
+      <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>2</v>
       </c>
+      <c r="B8" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>3</v>
       </c>
+      <c r="B9" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -585,16 +601,25 @@
       <c r="A12" t="s">
         <v>6</v>
       </c>
+      <c r="B12" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>7</v>
       </c>
+      <c r="B13" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>8</v>
       </c>
+      <c r="B14" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -606,49 +631,55 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B18" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="B21" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
         <v>18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>